<commit_message>
fix for openstreetmap and add browserstack config
</commit_message>
<xml_diff>
--- a/testdata/Company.xlsx
+++ b/testdata/Company.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Sales Force\Automation\stp-automation-test\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Sales Force\Automation\sales-force-automation-test\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE4BA64F-8184-41DD-949E-2C7E1557BEA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE733798-1BEF-4E2C-8D99-F352C8EF4DBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C7681F3F-D0BE-43DE-AC81-0EAE175E5E0E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C7681F3F-D0BE-43DE-AC81-0EAE175E5E0E}"/>
   </bookViews>
   <sheets>
     <sheet name="addCompany" sheetId="3" r:id="rId1"/>
@@ -34,8 +34,42 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Fendy Ridwan</author>
+  </authors>
+  <commentList>
+    <comment ref="F2" authorId="0" shapeId="0" xr:uid="{43A45A2D-3156-48D3-ABFE-AFECE5C7D017}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Fendy Ridwan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+googlemap or openstreetmap</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="29">
   <si>
     <t>expectedResult</t>
   </si>
@@ -119,13 +153,16 @@
   </si>
   <si>
     <t>This company was successfully updated</t>
+  </si>
+  <si>
+    <t>openstreetmap</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -151,6 +188,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -628,7 +678,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B86591FD-2F75-473D-9D49-464CBC030A17}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B86591FD-2F75-473D-9D49-464CBC030A17}">
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -697,7 +747,7 @@
         <v>15</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>19</v>
@@ -718,5 +768,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>